<commit_message>
nuevos cambios en contralor, modelo y vista
</commit_message>
<xml_diff>
--- a/myapp/src/main/resources/plantilla1.xlsx
+++ b/myapp/src/main/resources/plantilla1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\App_TecnoMat\app_lectorArchivos\myapp\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6D06A9-CABB-423C-8ECD-114E78B83700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9FF906-8C9B-4692-9128-0C081BE1E765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{501981FC-E882-4770-BB78-4C8F6F42D128}"/>
+    <workbookView xWindow="5130" yWindow="3165" windowWidth="21600" windowHeight="11385" xr2:uid="{501981FC-E882-4770-BB78-4C8F6F42D128}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -503,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -582,16 +582,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -602,35 +592,41 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -964,7 +960,6 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="8"/>
-      <c r="L1" s="33"/>
       <c r="M1" s="24"/>
     </row>
     <row r="2" spans="1:13" ht="26.25" x14ac:dyDescent="0.25">
@@ -973,16 +968,15 @@
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
-      <c r="D2" s="32" t="s">
+      <c r="D2" s="46" t="s">
         <v>67</v>
       </c>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
       <c r="J2" s="8"/>
-      <c r="L2" s="33"/>
       <c r="M2" s="25"/>
     </row>
     <row r="3" spans="1:13" ht="18" x14ac:dyDescent="0.25">
@@ -998,7 +992,6 @@
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
       <c r="J3" s="23"/>
-      <c r="L3" s="33"/>
       <c r="M3" s="25"/>
     </row>
     <row r="4" spans="1:13" ht="18" x14ac:dyDescent="0.25">
@@ -1018,7 +1011,6 @@
       <c r="H4" s="6"/>
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
-      <c r="L4" s="33"/>
       <c r="M4" s="25"/>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.25">
@@ -1036,15 +1028,15 @@
       <c r="F5" s="6"/>
       <c r="G5" s="26"/>
       <c r="H5" s="26"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="44" t="s">
+      <c r="I5" s="13"/>
+      <c r="J5" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="K5" s="44"/>
-      <c r="L5" s="30" t="s">
+      <c r="K5" s="43"/>
+      <c r="L5" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="38"/>
+      <c r="M5" s="39"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
@@ -1054,22 +1046,22 @@
       <c r="C6" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="E6" s="31"/>
+      <c r="E6" s="42"/>
       <c r="F6" s="6"/>
       <c r="G6" s="27"/>
       <c r="H6" s="27"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="45" t="s">
+      <c r="I6" s="34"/>
+      <c r="J6" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="K6" s="45"/>
-      <c r="L6" s="42">
+      <c r="K6" s="44"/>
+      <c r="L6" s="40">
         <v>46065</v>
       </c>
-      <c r="M6" s="39"/>
+      <c r="M6" s="41"/>
     </row>
     <row r="7" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
@@ -1080,21 +1072,21 @@
       <c r="F7" s="6"/>
       <c r="G7" s="28"/>
       <c r="H7" s="28"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="46" t="s">
+      <c r="I7" s="34"/>
+      <c r="J7" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="K7" s="46"/>
-      <c r="L7" s="42">
+      <c r="K7" s="45"/>
+      <c r="L7" s="40">
         <v>46072</v>
       </c>
-      <c r="M7" s="39"/>
+      <c r="M7" s="41"/>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="37"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
       <c r="E8" s="17"/>
@@ -1102,35 +1094,29 @@
       <c r="G8" s="18"/>
       <c r="H8" s="18"/>
       <c r="I8" s="18"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="47"/>
-      <c r="L8" s="33"/>
+      <c r="J8" s="35"/>
+      <c r="K8" s="36"/>
       <c r="M8" s="25"/>
     </row>
     <row r="9" spans="1:13" ht="24" x14ac:dyDescent="0.25">
-      <c r="A9" s="35" t="s">
+      <c r="A9" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="35" t="s">
+      <c r="C9" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="36" t="s">
+      <c r="E9" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="34"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="48"/>
-      <c r="M9" s="48"/>
+      <c r="F9" s="30"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
@@ -2014,14 +2000,14 @@
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="L7:M7"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D2:I2"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="L7:M7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>